<commit_message>
inflation first with result
</commit_message>
<xml_diff>
--- a/data/inner_join.xlsx
+++ b/data/inner_join.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R209"/>
+  <dimension ref="A1:S209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +523,11 @@
           <t>cfaFr</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -583,6 +592,9 @@
       <c r="R2" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="S2" s="2" t="n">
+        <v>44287</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -647,6 +659,9 @@
       <c r="R3" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="S3" s="2" t="n">
+        <v>44256</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -711,6 +726,9 @@
       <c r="R4" t="n">
         <v>0.7</v>
       </c>
+      <c r="S4" s="2" t="n">
+        <v>44228</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -775,6 +793,9 @@
       <c r="R5" t="n">
         <v>0.71</v>
       </c>
+      <c r="S5" s="2" t="n">
+        <v>44197</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -839,6 +860,9 @@
       <c r="R6" t="n">
         <v>0.7</v>
       </c>
+      <c r="S6" s="2" t="n">
+        <v>44166</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -903,6 +927,9 @@
       <c r="R7" t="n">
         <v>0.68</v>
       </c>
+      <c r="S7" s="2" t="n">
+        <v>44136</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -967,6 +994,9 @@
       <c r="R8" t="n">
         <v>0.68</v>
       </c>
+      <c r="S8" s="2" t="n">
+        <v>44105</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1031,6 +1061,9 @@
       <c r="R9" t="n">
         <v>0.68</v>
       </c>
+      <c r="S9" s="2" t="n">
+        <v>44075</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1095,6 +1128,9 @@
       <c r="R10" t="n">
         <v>0.66</v>
       </c>
+      <c r="S10" s="2" t="n">
+        <v>44044</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1159,6 +1195,9 @@
       <c r="R11" t="n">
         <v>0.53</v>
       </c>
+      <c r="S11" s="2" t="n">
+        <v>44013</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1223,6 +1262,9 @@
       <c r="R12" t="n">
         <v>0.53</v>
       </c>
+      <c r="S12" s="2" t="n">
+        <v>43983</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1287,6 +1329,9 @@
       <c r="R13" t="n">
         <v>0.51</v>
       </c>
+      <c r="S13" s="2" t="n">
+        <v>43952</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1351,6 +1396,9 @@
       <c r="R14" t="n">
         <v>0.51</v>
       </c>
+      <c r="S14" s="2" t="n">
+        <v>43922</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1415,6 +1463,9 @@
       <c r="R15" t="n">
         <v>0.52</v>
       </c>
+      <c r="S15" s="2" t="n">
+        <v>43891</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1479,6 +1530,9 @@
       <c r="R16" t="n">
         <v>0.5</v>
       </c>
+      <c r="S16" s="2" t="n">
+        <v>43862</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1543,6 +1597,9 @@
       <c r="R17" t="n">
         <v>0.52</v>
       </c>
+      <c r="S17" s="2" t="n">
+        <v>43831</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1607,6 +1664,9 @@
       <c r="R18" t="n">
         <v>0.52</v>
       </c>
+      <c r="S18" s="2" t="n">
+        <v>43800</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1671,6 +1731,9 @@
       <c r="R19" t="n">
         <v>0.52</v>
       </c>
+      <c r="S19" s="2" t="n">
+        <v>43770</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1735,6 +1798,9 @@
       <c r="R20" t="n">
         <v>0.52</v>
       </c>
+      <c r="S20" s="2" t="n">
+        <v>43739</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1799,6 +1865,9 @@
       <c r="R21" t="n">
         <v>0.51</v>
       </c>
+      <c r="S21" s="2" t="n">
+        <v>43709</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1863,6 +1932,9 @@
       <c r="R22" t="n">
         <v>0.52</v>
       </c>
+      <c r="S22" s="2" t="n">
+        <v>43678</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1927,6 +1999,9 @@
       <c r="R23" t="n">
         <v>0.53</v>
       </c>
+      <c r="S23" s="2" t="n">
+        <v>43647</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1991,6 +2066,9 @@
       <c r="R24" t="n">
         <v>0.53</v>
       </c>
+      <c r="S24" s="2" t="n">
+        <v>43617</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2055,6 +2133,9 @@
       <c r="R25" t="n">
         <v>0.52</v>
       </c>
+      <c r="S25" s="2" t="n">
+        <v>43586</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2119,6 +2200,9 @@
       <c r="R26" t="n">
         <v>0.53</v>
       </c>
+      <c r="S26" s="2" t="n">
+        <v>43556</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2183,6 +2267,9 @@
       <c r="R27" t="n">
         <v>0.53</v>
       </c>
+      <c r="S27" s="2" t="n">
+        <v>43525</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2247,6 +2334,9 @@
       <c r="R28" t="n">
         <v>0.53</v>
       </c>
+      <c r="S28" s="2" t="n">
+        <v>43497</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2311,6 +2401,9 @@
       <c r="R29" t="n">
         <v>0.53</v>
       </c>
+      <c r="S29" s="2" t="n">
+        <v>43466</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2375,6 +2468,9 @@
       <c r="R30" t="n">
         <v>0.53</v>
       </c>
+      <c r="S30" s="2" t="n">
+        <v>43435</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2439,6 +2535,9 @@
       <c r="R31" t="n">
         <v>0.53</v>
       </c>
+      <c r="S31" s="2" t="n">
+        <v>43405</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2503,6 +2602,9 @@
       <c r="R32" t="n">
         <v>0.54</v>
       </c>
+      <c r="S32" s="2" t="n">
+        <v>43374</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2567,6 +2669,9 @@
       <c r="R33" t="n">
         <v>0.54</v>
       </c>
+      <c r="S33" s="2" t="n">
+        <v>43344</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2631,6 +2736,9 @@
       <c r="R34" t="n">
         <v>0.54</v>
       </c>
+      <c r="S34" s="2" t="n">
+        <v>43313</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2695,6 +2803,9 @@
       <c r="R35" t="n">
         <v>0.54</v>
       </c>
+      <c r="S35" s="2" t="n">
+        <v>43282</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2759,6 +2870,9 @@
       <c r="R36" t="n">
         <v>0.54</v>
       </c>
+      <c r="S36" s="2" t="n">
+        <v>43252</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2823,6 +2937,9 @@
       <c r="R37" t="n">
         <v>0.55</v>
       </c>
+      <c r="S37" s="2" t="n">
+        <v>43221</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2887,6 +3004,9 @@
       <c r="R38" t="n">
         <v>0.57</v>
       </c>
+      <c r="S38" s="2" t="n">
+        <v>43191</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2951,6 +3071,9 @@
       <c r="R39" t="n">
         <v>0.57</v>
       </c>
+      <c r="S39" s="2" t="n">
+        <v>43160</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3015,6 +3138,9 @@
       <c r="R40" t="n">
         <v>0.58</v>
       </c>
+      <c r="S40" s="2" t="n">
+        <v>43132</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3079,6 +3205,9 @@
       <c r="R41" t="n">
         <v>0.57</v>
       </c>
+      <c r="S41" s="2" t="n">
+        <v>43101</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3143,6 +3272,9 @@
       <c r="R42" t="n">
         <v>0.55</v>
       </c>
+      <c r="S42" s="2" t="n">
+        <v>43070</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3207,6 +3339,9 @@
       <c r="R43" t="n">
         <v>0.54</v>
       </c>
+      <c r="S43" s="2" t="n">
+        <v>43040</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3271,6 +3406,9 @@
       <c r="R44" t="n">
         <v>0.55</v>
       </c>
+      <c r="S44" s="2" t="n">
+        <v>43009</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3335,6 +3473,9 @@
       <c r="R45" t="n">
         <v>0.5600000000000001</v>
       </c>
+      <c r="S45" s="2" t="n">
+        <v>42979</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3399,6 +3540,9 @@
       <c r="R46" t="n">
         <v>0.55</v>
       </c>
+      <c r="S46" s="2" t="n">
+        <v>42948</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3463,6 +3607,9 @@
       <c r="R47" t="n">
         <v>0.54</v>
       </c>
+      <c r="S47" s="2" t="n">
+        <v>42917</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3527,6 +3674,9 @@
       <c r="R48" t="n">
         <v>0.52</v>
       </c>
+      <c r="S48" s="2" t="n">
+        <v>42887</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3591,6 +3741,9 @@
       <c r="R49" t="n">
         <v>0.51</v>
       </c>
+      <c r="S49" s="2" t="n">
+        <v>42856</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3655,6 +3808,9 @@
       <c r="R50" t="n">
         <v>0.5</v>
       </c>
+      <c r="S50" s="2" t="n">
+        <v>42826</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3719,6 +3875,9 @@
       <c r="R51" t="n">
         <v>0.5</v>
       </c>
+      <c r="S51" s="2" t="n">
+        <v>42795</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3783,6 +3942,9 @@
       <c r="R52" t="n">
         <v>0.5</v>
       </c>
+      <c r="S52" s="2" t="n">
+        <v>42767</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3847,6 +4009,9 @@
       <c r="R53" t="n">
         <v>0.49</v>
       </c>
+      <c r="S53" s="2" t="n">
+        <v>42736</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3911,6 +4076,9 @@
       <c r="R54" t="n">
         <v>0.47</v>
       </c>
+      <c r="S54" s="2" t="n">
+        <v>42705</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3975,6 +4143,9 @@
       <c r="R55" t="n">
         <v>0.5</v>
       </c>
+      <c r="S55" s="2" t="n">
+        <v>42675</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4039,6 +4210,9 @@
       <c r="R56" t="n">
         <v>0.51</v>
       </c>
+      <c r="S56" s="2" t="n">
+        <v>42644</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4103,6 +4277,9 @@
       <c r="R57" t="n">
         <v>0.52</v>
       </c>
+      <c r="S57" s="2" t="n">
+        <v>42614</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4167,6 +4344,9 @@
       <c r="R58" t="n">
         <v>0.53</v>
       </c>
+      <c r="S58" s="2" t="n">
+        <v>42583</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4231,6 +4411,9 @@
       <c r="R59" t="n">
         <v>0.49</v>
       </c>
+      <c r="S59" s="2" t="n">
+        <v>42552</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4295,6 +4478,9 @@
       <c r="R60" t="n">
         <v>0.38</v>
       </c>
+      <c r="S60" s="2" t="n">
+        <v>42522</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4359,6 +4545,9 @@
       <c r="R61" t="n">
         <v>0.34</v>
       </c>
+      <c r="S61" s="2" t="n">
+        <v>42491</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4423,6 +4612,9 @@
       <c r="R62" t="n">
         <v>0.34</v>
       </c>
+      <c r="S62" s="2" t="n">
+        <v>42461</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4487,6 +4679,9 @@
       <c r="R63" t="n">
         <v>0.33</v>
       </c>
+      <c r="S63" s="2" t="n">
+        <v>42430</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4551,6 +4746,9 @@
       <c r="R64" t="n">
         <v>0.33</v>
       </c>
+      <c r="S64" s="2" t="n">
+        <v>42401</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4615,6 +4813,9 @@
       <c r="R65" t="n">
         <v>0.33</v>
       </c>
+      <c r="S65" s="2" t="n">
+        <v>42370</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4679,6 +4880,9 @@
       <c r="R66" t="n">
         <v>0.32</v>
       </c>
+      <c r="S66" s="2" t="n">
+        <v>42339</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4743,6 +4947,9 @@
       <c r="R67" t="n">
         <v>0.32</v>
       </c>
+      <c r="S67" s="2" t="n">
+        <v>42309</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4807,6 +5014,9 @@
       <c r="R68" t="n">
         <v>0.34</v>
       </c>
+      <c r="S68" s="2" t="n">
+        <v>42278</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -4871,6 +5081,9 @@
       <c r="R69" t="n">
         <v>0.34</v>
       </c>
+      <c r="S69" s="2" t="n">
+        <v>42248</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -4935,6 +5148,9 @@
       <c r="R70" t="n">
         <v>0.33</v>
       </c>
+      <c r="S70" s="2" t="n">
+        <v>42217</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -4999,6 +5215,9 @@
       <c r="R71" t="n">
         <v>0.33</v>
       </c>
+      <c r="S71" s="2" t="n">
+        <v>42186</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -5063,6 +5282,9 @@
       <c r="R72" t="n">
         <v>0.34</v>
       </c>
+      <c r="S72" s="2" t="n">
+        <v>42156</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -5127,6 +5349,9 @@
       <c r="R73" t="n">
         <v>0.34</v>
       </c>
+      <c r="S73" s="2" t="n">
+        <v>42125</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -5191,6 +5416,9 @@
       <c r="R74" t="n">
         <v>0.32</v>
       </c>
+      <c r="S74" s="2" t="n">
+        <v>42095</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -5255,6 +5483,9 @@
       <c r="R75" t="n">
         <v>0.32</v>
       </c>
+      <c r="S75" s="2" t="n">
+        <v>42064</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -5319,6 +5550,9 @@
       <c r="R76" t="n">
         <v>0.31</v>
       </c>
+      <c r="S76" s="2" t="n">
+        <v>42036</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5383,6 +5617,9 @@
       <c r="R77" t="n">
         <v>0.3</v>
       </c>
+      <c r="S77" s="2" t="n">
+        <v>42005</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -5447,6 +5684,9 @@
       <c r="R78" t="n">
         <v>0.32</v>
       </c>
+      <c r="S78" s="2" t="n">
+        <v>41974</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -5511,6 +5751,9 @@
       <c r="R79" t="n">
         <v>0.3</v>
       </c>
+      <c r="S79" s="2" t="n">
+        <v>41944</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -5575,6 +5818,9 @@
       <c r="R80" t="n">
         <v>0.3</v>
       </c>
+      <c r="S80" s="2" t="n">
+        <v>41913</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -5639,6 +5885,9 @@
       <c r="R81" t="n">
         <v>0.31</v>
       </c>
+      <c r="S81" s="2" t="n">
+        <v>41883</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -5703,6 +5952,9 @@
       <c r="R82" t="n">
         <v>0.32</v>
       </c>
+      <c r="S82" s="2" t="n">
+        <v>41852</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -5767,6 +6019,9 @@
       <c r="R83" t="n">
         <v>0.32</v>
       </c>
+      <c r="S83" s="2" t="n">
+        <v>41821</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -5831,6 +6086,9 @@
       <c r="R84" t="n">
         <v>0.32</v>
       </c>
+      <c r="S84" s="2" t="n">
+        <v>41791</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -5895,6 +6153,9 @@
       <c r="R85" t="n">
         <v>0.33</v>
       </c>
+      <c r="S85" s="2" t="n">
+        <v>41760</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -5959,6 +6220,9 @@
       <c r="R86" t="n">
         <v>0.33</v>
       </c>
+      <c r="S86" s="2" t="n">
+        <v>41730</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -6023,6 +6287,9 @@
       <c r="R87" t="n">
         <v>0.33</v>
       </c>
+      <c r="S87" s="2" t="n">
+        <v>41699</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -6087,6 +6354,9 @@
       <c r="R88" t="n">
         <v>0.32</v>
       </c>
+      <c r="S88" s="2" t="n">
+        <v>41671</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -6151,6 +6421,9 @@
       <c r="R89" t="n">
         <v>0.32</v>
       </c>
+      <c r="S89" s="2" t="n">
+        <v>41640</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -6215,6 +6488,9 @@
       <c r="R90" t="n">
         <v>0.32</v>
       </c>
+      <c r="S90" s="2" t="n">
+        <v>41609</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -6279,6 +6555,9 @@
       <c r="R91" t="n">
         <v>0.32</v>
       </c>
+      <c r="S91" s="2" t="n">
+        <v>41579</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -6343,6 +6622,9 @@
       <c r="R92" t="n">
         <v>0.32</v>
       </c>
+      <c r="S92" s="2" t="n">
+        <v>41548</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -6407,6 +6689,9 @@
       <c r="R93" t="n">
         <v>0.32</v>
       </c>
+      <c r="S93" s="2" t="n">
+        <v>41518</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -6471,6 +6756,9 @@
       <c r="R94" t="n">
         <v>0.31</v>
       </c>
+      <c r="S94" s="2" t="n">
+        <v>41487</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -6535,6 +6823,9 @@
       <c r="R95" t="n">
         <v>0.3</v>
       </c>
+      <c r="S95" s="2" t="n">
+        <v>41456</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -6599,6 +6890,9 @@
       <c r="R96" t="n">
         <v>0.31</v>
       </c>
+      <c r="S96" s="2" t="n">
+        <v>41426</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -6663,6 +6957,9 @@
       <c r="R97" t="n">
         <v>0.31</v>
       </c>
+      <c r="S97" s="2" t="n">
+        <v>41395</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -6727,6 +7024,9 @@
       <c r="R98" t="n">
         <v>0.31</v>
       </c>
+      <c r="S98" s="2" t="n">
+        <v>41365</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -6791,6 +7091,9 @@
       <c r="R99" t="n">
         <v>0.31</v>
       </c>
+      <c r="S99" s="2" t="n">
+        <v>41334</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -6855,6 +7158,9 @@
       <c r="R100" t="n">
         <v>0.32</v>
       </c>
+      <c r="S100" s="2" t="n">
+        <v>41306</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -6919,6 +7225,9 @@
       <c r="R101" t="n">
         <v>0.31</v>
       </c>
+      <c r="S101" s="2" t="n">
+        <v>41275</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -6983,6 +7292,9 @@
       <c r="R102" t="n">
         <v>0.31</v>
       </c>
+      <c r="S102" s="2" t="n">
+        <v>41244</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -7047,6 +7359,9 @@
       <c r="R103" t="n">
         <v>0.3</v>
       </c>
+      <c r="S103" s="2" t="n">
+        <v>41214</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -7111,6 +7426,9 @@
       <c r="R104" t="n">
         <v>0.31</v>
       </c>
+      <c r="S104" s="2" t="n">
+        <v>41183</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -7175,6 +7493,9 @@
       <c r="R105" t="n">
         <v>0.3</v>
       </c>
+      <c r="S105" s="2" t="n">
+        <v>41153</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -7239,6 +7560,9 @@
       <c r="R106" t="n">
         <v>0.29</v>
       </c>
+      <c r="S106" s="2" t="n">
+        <v>41122</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -7303,6 +7627,9 @@
       <c r="R107" t="n">
         <v>0.29</v>
       </c>
+      <c r="S107" s="2" t="n">
+        <v>41091</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -7367,6 +7694,9 @@
       <c r="R108" t="n">
         <v>0.3</v>
       </c>
+      <c r="S108" s="2" t="n">
+        <v>41061</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -7431,6 +7761,9 @@
       <c r="R109" t="n">
         <v>0.3</v>
       </c>
+      <c r="S109" s="2" t="n">
+        <v>41030</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -7495,6 +7828,9 @@
       <c r="R110" t="n">
         <v>0.31</v>
       </c>
+      <c r="S110" s="2" t="n">
+        <v>41000</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -7559,6 +7895,9 @@
       <c r="R111" t="n">
         <v>0.31</v>
       </c>
+      <c r="S111" s="2" t="n">
+        <v>40969</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -7623,6 +7962,9 @@
       <c r="R112" t="n">
         <v>0.31</v>
       </c>
+      <c r="S112" s="2" t="n">
+        <v>40940</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -7687,6 +8029,9 @@
       <c r="R113" t="n">
         <v>0.31</v>
       </c>
+      <c r="S113" s="2" t="n">
+        <v>40909</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -7751,6 +8096,9 @@
       <c r="R114" t="n">
         <v>0.31</v>
       </c>
+      <c r="S114" s="2" t="n">
+        <v>40878</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -7815,6 +8163,9 @@
       <c r="R115" t="n">
         <v>0.32</v>
       </c>
+      <c r="S115" s="2" t="n">
+        <v>40848</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -7879,6 +8230,9 @@
       <c r="R116" t="n">
         <v>0.32</v>
       </c>
+      <c r="S116" s="2" t="n">
+        <v>40817</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -7943,6 +8297,9 @@
       <c r="R117" t="n">
         <v>0.32</v>
       </c>
+      <c r="S117" s="2" t="n">
+        <v>40787</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -8007,6 +8364,9 @@
       <c r="R118" t="n">
         <v>0.33</v>
       </c>
+      <c r="S118" s="2" t="n">
+        <v>40756</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -8071,6 +8431,9 @@
       <c r="R119" t="n">
         <v>0.33</v>
       </c>
+      <c r="S119" s="2" t="n">
+        <v>40725</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -8135,6 +8498,9 @@
       <c r="R120" t="n">
         <v>0.34</v>
       </c>
+      <c r="S120" s="2" t="n">
+        <v>40695</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -8199,6 +8565,9 @@
       <c r="R121" t="n">
         <v>0.33</v>
       </c>
+      <c r="S121" s="2" t="n">
+        <v>40664</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -8263,6 +8632,9 @@
       <c r="R122" t="n">
         <v>0.33</v>
       </c>
+      <c r="S122" s="2" t="n">
+        <v>40634</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -8327,6 +8699,9 @@
       <c r="R123" t="n">
         <v>0.32</v>
       </c>
+      <c r="S123" s="2" t="n">
+        <v>40603</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -8391,6 +8766,9 @@
       <c r="R124" t="n">
         <v>0.31</v>
       </c>
+      <c r="S124" s="2" t="n">
+        <v>40575</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -8455,6 +8833,9 @@
       <c r="R125" t="n">
         <v>0.3</v>
       </c>
+      <c r="S125" s="2" t="n">
+        <v>40544</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -8519,6 +8900,9 @@
       <c r="R126" t="n">
         <v>0.3</v>
       </c>
+      <c r="S126" s="2" t="n">
+        <v>40513</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -8583,6 +8967,9 @@
       <c r="R127" t="n">
         <v>0.31</v>
       </c>
+      <c r="S127" s="2" t="n">
+        <v>40483</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -8647,6 +9034,9 @@
       <c r="R128" t="n">
         <v>0.32</v>
       </c>
+      <c r="S128" s="2" t="n">
+        <v>40452</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -8711,6 +9101,9 @@
       <c r="R129" t="n">
         <v>0.3</v>
       </c>
+      <c r="S129" s="2" t="n">
+        <v>40422</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -8775,6 +9168,9 @@
       <c r="R130" t="n">
         <v>0.29</v>
       </c>
+      <c r="S130" s="2" t="n">
+        <v>40391</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -8839,6 +9235,9 @@
       <c r="R131" t="n">
         <v>0.29</v>
       </c>
+      <c r="S131" s="2" t="n">
+        <v>40360</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -8903,6 +9302,9 @@
       <c r="R132" t="n">
         <v>0.28</v>
       </c>
+      <c r="S132" s="2" t="n">
+        <v>40330</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -8967,6 +9369,9 @@
       <c r="R133" t="n">
         <v>0.28</v>
       </c>
+      <c r="S133" s="2" t="n">
+        <v>40299</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -9031,6 +9436,9 @@
       <c r="R134" t="n">
         <v>0.28</v>
       </c>
+      <c r="S134" s="2" t="n">
+        <v>40269</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -9095,6 +9503,9 @@
       <c r="R135" t="n">
         <v>0.31</v>
       </c>
+      <c r="S135" s="2" t="n">
+        <v>40238</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -9159,6 +9570,9 @@
       <c r="R136" t="n">
         <v>0.31</v>
       </c>
+      <c r="S136" s="2" t="n">
+        <v>40210</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -9223,6 +9637,9 @@
       <c r="R137" t="n">
         <v>0.32</v>
       </c>
+      <c r="S137" s="2" t="n">
+        <v>40179</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -9287,6 +9704,9 @@
       <c r="R138" t="n">
         <v>0.33</v>
       </c>
+      <c r="S138" s="2" t="n">
+        <v>40148</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -9351,6 +9771,9 @@
       <c r="R139" t="n">
         <v>0.34</v>
       </c>
+      <c r="S139" s="2" t="n">
+        <v>40118</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -9415,6 +9838,9 @@
       <c r="R140" t="n">
         <v>0.33</v>
       </c>
+      <c r="S140" s="2" t="n">
+        <v>40087</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -9479,6 +9905,9 @@
       <c r="R141" t="n">
         <v>0.33</v>
       </c>
+      <c r="S141" s="2" t="n">
+        <v>40057</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -9543,6 +9972,9 @@
       <c r="R142" t="n">
         <v>0.36</v>
       </c>
+      <c r="S142" s="2" t="n">
+        <v>40026</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -9607,6 +10039,9 @@
       <c r="R143" t="n">
         <v>0.32</v>
       </c>
+      <c r="S143" s="2" t="n">
+        <v>39995</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -9671,6 +10106,9 @@
       <c r="R144" t="n">
         <v>0.31</v>
       </c>
+      <c r="S144" s="2" t="n">
+        <v>39965</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -9735,6 +10173,9 @@
       <c r="R145" t="n">
         <v>0.3</v>
       </c>
+      <c r="S145" s="2" t="n">
+        <v>39934</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -9799,6 +10240,9 @@
       <c r="R146" t="n">
         <v>0.29</v>
       </c>
+      <c r="S146" s="2" t="n">
+        <v>39904</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -9863,6 +10307,9 @@
       <c r="R147" t="n">
         <v>0.29</v>
       </c>
+      <c r="S147" s="2" t="n">
+        <v>39873</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -9927,6 +10374,9 @@
       <c r="R148" t="n">
         <v>0.28</v>
       </c>
+      <c r="S148" s="2" t="n">
+        <v>39845</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -9991,6 +10441,9 @@
       <c r="R149" t="n">
         <v>0.29</v>
       </c>
+      <c r="S149" s="2" t="n">
+        <v>39814</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -10055,6 +10508,9 @@
       <c r="R150" t="n">
         <v>0.26</v>
       </c>
+      <c r="S150" s="2" t="n">
+        <v>39783</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -10119,6 +10575,9 @@
       <c r="R151" t="n">
         <v>0.23</v>
       </c>
+      <c r="S151" s="2" t="n">
+        <v>39753</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -10183,6 +10642,9 @@
       <c r="R152" t="n">
         <v>0.24</v>
       </c>
+      <c r="S152" s="2" t="n">
+        <v>39722</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -10247,6 +10709,9 @@
       <c r="R153" t="n">
         <v>0.26</v>
       </c>
+      <c r="S153" s="2" t="n">
+        <v>39692</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -10311,6 +10776,9 @@
       <c r="R154" t="n">
         <v>0.27</v>
       </c>
+      <c r="S154" s="2" t="n">
+        <v>39661</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -10375,6 +10843,9 @@
       <c r="R155" t="n">
         <v>0.28</v>
       </c>
+      <c r="S155" s="2" t="n">
+        <v>39630</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -10439,6 +10910,9 @@
       <c r="R156" t="n">
         <v>0.27</v>
       </c>
+      <c r="S156" s="2" t="n">
+        <v>39600</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -10503,6 +10977,9 @@
       <c r="R157" t="n">
         <v>0.28</v>
       </c>
+      <c r="S157" s="2" t="n">
+        <v>39569</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -10567,6 +11044,9 @@
       <c r="R158" t="n">
         <v>0.28</v>
       </c>
+      <c r="S158" s="2" t="n">
+        <v>39539</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -10631,6 +11111,9 @@
       <c r="R159" t="n">
         <v>0.27</v>
       </c>
+      <c r="S159" s="2" t="n">
+        <v>39508</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -10695,6 +11178,9 @@
       <c r="R160" t="n">
         <v>0.26</v>
       </c>
+      <c r="S160" s="2" t="n">
+        <v>39479</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -10759,6 +11245,9 @@
       <c r="R161" t="n">
         <v>0.26</v>
       </c>
+      <c r="S161" s="2" t="n">
+        <v>39448</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -10823,6 +11312,9 @@
       <c r="R162" t="n">
         <v>0.26</v>
       </c>
+      <c r="S162" s="2" t="n">
+        <v>39417</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -10887,6 +11379,9 @@
       <c r="R163" t="n">
         <v>0.26</v>
       </c>
+      <c r="S163" s="2" t="n">
+        <v>39387</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -10951,6 +11446,9 @@
       <c r="R164" t="n">
         <v>0.27</v>
       </c>
+      <c r="S164" s="2" t="n">
+        <v>39356</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -11015,6 +11513,9 @@
       <c r="R165" t="n">
         <v>0.26</v>
       </c>
+      <c r="S165" s="2" t="n">
+        <v>39326</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -11079,6 +11580,9 @@
       <c r="R166" t="n">
         <v>0.26</v>
       </c>
+      <c r="S166" s="2" t="n">
+        <v>39295</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -11143,6 +11647,9 @@
       <c r="R167" t="n">
         <v>0.26</v>
       </c>
+      <c r="S167" s="2" t="n">
+        <v>39264</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -11207,6 +11714,9 @@
       <c r="R168" t="n">
         <v>0.26</v>
       </c>
+      <c r="S168" s="2" t="n">
+        <v>39234</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -11271,6 +11781,9 @@
       <c r="R169" t="n">
         <v>0.25</v>
       </c>
+      <c r="S169" s="2" t="n">
+        <v>39203</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -11335,6 +11848,9 @@
       <c r="R170" t="n">
         <v>0.26</v>
       </c>
+      <c r="S170" s="2" t="n">
+        <v>39173</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -11399,6 +11915,9 @@
       <c r="R171" t="n">
         <v>0.25</v>
       </c>
+      <c r="S171" s="2" t="n">
+        <v>39142</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -11463,6 +11982,9 @@
       <c r="R172" t="n">
         <v>0.24</v>
       </c>
+      <c r="S172" s="2" t="n">
+        <v>39114</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -11527,6 +12049,9 @@
       <c r="R173" t="n">
         <v>0.25</v>
       </c>
+      <c r="S173" s="2" t="n">
+        <v>39083</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -11591,6 +12116,9 @@
       <c r="R174" t="n">
         <v>0.24</v>
       </c>
+      <c r="S174" s="2" t="n">
+        <v>39052</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -11655,6 +12183,9 @@
       <c r="R175" t="n">
         <v>0.25</v>
       </c>
+      <c r="S175" s="2" t="n">
+        <v>39022</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -11719,6 +12250,9 @@
       <c r="R176" t="n">
         <v>0.25</v>
       </c>
+      <c r="S176" s="2" t="n">
+        <v>38991</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -11783,6 +12317,9 @@
       <c r="R177" t="n">
         <v>0.25</v>
       </c>
+      <c r="S177" s="2" t="n">
+        <v>38961</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -11847,6 +12384,9 @@
       <c r="R178" t="n">
         <v>0.25</v>
       </c>
+      <c r="S178" s="2" t="n">
+        <v>38930</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -11911,6 +12451,9 @@
       <c r="R179" t="n">
         <v>0.24</v>
       </c>
+      <c r="S179" s="2" t="n">
+        <v>38899</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -11975,6 +12518,9 @@
       <c r="R180" t="n">
         <v>0.24</v>
       </c>
+      <c r="S180" s="2" t="n">
+        <v>38869</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -12039,6 +12585,9 @@
       <c r="R181" t="n">
         <v>0.25</v>
       </c>
+      <c r="S181" s="2" t="n">
+        <v>38838</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -12103,6 +12652,9 @@
       <c r="R182" t="n">
         <v>0.24</v>
       </c>
+      <c r="S182" s="2" t="n">
+        <v>38808</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -12167,6 +12719,9 @@
       <c r="R183" t="n">
         <v>0.23</v>
       </c>
+      <c r="S183" s="2" t="n">
+        <v>38777</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -12231,6 +12786,9 @@
       <c r="R184" t="n">
         <v>0.23</v>
       </c>
+      <c r="S184" s="2" t="n">
+        <v>38749</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -12295,6 +12853,9 @@
       <c r="R185" t="n">
         <v>0.24</v>
       </c>
+      <c r="S185" s="2" t="n">
+        <v>38718</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -12359,6 +12920,9 @@
       <c r="R186" t="n">
         <v>0.23</v>
       </c>
+      <c r="S186" s="2" t="n">
+        <v>38687</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -12423,6 +12987,9 @@
       <c r="R187" t="n">
         <v>0.23</v>
       </c>
+      <c r="S187" s="2" t="n">
+        <v>38657</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -12487,6 +13054,9 @@
       <c r="R188" t="n">
         <v>0.24</v>
       </c>
+      <c r="S188" s="2" t="n">
+        <v>38626</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -12551,6 +13121,9 @@
       <c r="R189" t="n">
         <v>0.24</v>
       </c>
+      <c r="S189" s="2" t="n">
+        <v>38596</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -12615,6 +13188,9 @@
       <c r="R190" t="n">
         <v>0.25</v>
       </c>
+      <c r="S190" s="2" t="n">
+        <v>38565</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -12679,6 +13255,9 @@
       <c r="R191" t="n">
         <v>0.24</v>
       </c>
+      <c r="S191" s="2" t="n">
+        <v>38534</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -12743,6 +13322,9 @@
       <c r="R192" t="n">
         <v>0.25</v>
       </c>
+      <c r="S192" s="2" t="n">
+        <v>38504</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -12807,6 +13389,9 @@
       <c r="R193" t="n">
         <v>0.26</v>
       </c>
+      <c r="S193" s="2" t="n">
+        <v>38473</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -12871,6 +13456,9 @@
       <c r="R194" t="n">
         <v>0.26</v>
       </c>
+      <c r="S194" s="2" t="n">
+        <v>38443</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -12935,6 +13523,9 @@
       <c r="R195" t="n">
         <v>0.27</v>
       </c>
+      <c r="S195" s="2" t="n">
+        <v>38412</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -12999,6 +13590,9 @@
       <c r="R196" t="n">
         <v>0.26</v>
       </c>
+      <c r="S196" s="2" t="n">
+        <v>38384</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -13063,6 +13657,9 @@
       <c r="R197" t="n">
         <v>0.27</v>
       </c>
+      <c r="S197" s="2" t="n">
+        <v>38353</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -13127,6 +13724,9 @@
       <c r="R198" t="n">
         <v>0.27</v>
       </c>
+      <c r="S198" s="2" t="n">
+        <v>38322</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -13191,6 +13791,9 @@
       <c r="R199" t="n">
         <v>0.26</v>
       </c>
+      <c r="S199" s="2" t="n">
+        <v>38292</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -13255,6 +13858,9 @@
       <c r="R200" t="n">
         <v>0.25</v>
       </c>
+      <c r="S200" s="2" t="n">
+        <v>38261</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -13319,6 +13925,9 @@
       <c r="R201" t="n">
         <v>0.25</v>
       </c>
+      <c r="S201" s="2" t="n">
+        <v>38231</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -13383,6 +13992,9 @@
       <c r="R202" t="n">
         <v>0.25</v>
       </c>
+      <c r="S202" s="2" t="n">
+        <v>38200</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -13447,6 +14059,9 @@
       <c r="R203" t="n">
         <v>0.25</v>
       </c>
+      <c r="S203" s="2" t="n">
+        <v>38169</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -13511,6 +14126,9 @@
       <c r="R204" t="n">
         <v>0.24</v>
       </c>
+      <c r="S204" s="2" t="n">
+        <v>38139</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -13575,6 +14193,9 @@
       <c r="R205" t="n">
         <v>0.24</v>
       </c>
+      <c r="S205" s="2" t="n">
+        <v>38108</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -13639,6 +14260,9 @@
       <c r="R206" t="n">
         <v>0.24</v>
       </c>
+      <c r="S206" s="2" t="n">
+        <v>38078</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -13703,6 +14327,9 @@
       <c r="R207" t="n">
         <v>0.25</v>
       </c>
+      <c r="S207" s="2" t="n">
+        <v>38047</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -13767,6 +14394,9 @@
       <c r="R208" t="n">
         <v>0.2</v>
       </c>
+      <c r="S208" s="2" t="n">
+        <v>38018</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -13830,6 +14460,9 @@
       </c>
       <c r="R209" t="n">
         <v>0.16</v>
+      </c>
+      <c r="S209" s="2" t="n">
+        <v>37987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>